<commit_message>
Merge invoicing-through-production, add month-end close and RACI owners
- Collapse Invoicing/Coil Inward/Slitting/Production into one step
  (Invoicing -> Production), keeping each sub-step's own detail and
  System/Software value.
- Add Month-End Reconciliation & Settlement as the closing step
  (Siddharth; Excel for the FIFO/thickness close, Zoho Books for
  Net CN/DN settlement).
- Fold in the team's responsibility/RACI sheet: named owners for
  Campaign Planning, RM Opportunity, Order Creation, and Material
  Readiness & Invoice Amount Check, plus two new steps inferred from
  it (Quality & Source Approval; CM Plant Contracting & Payment).
  Flags two open gaps: material ageing has no owner, and two roles
  (quality associate, Vinay) are still pending.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J9TXredfbUcJ8vSi96NRVo
</commit_message>
<xml_diff>
--- a/docs/PROCESS-MAP.xlsx
+++ b/docs/PROCESS-MAP.xlsx
@@ -528,13 +528,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -547,7 +547,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>RM Opportunity (SFDC) through Dispatch/Sales, plus Campaign Planning &amp; Monitoring. Yellow = to be filled in by process owners.</t>
+          <t>Campaign Planning through month-end close. Yellow = to be filled in by process owners.</t>
         </is>
       </c>
     </row>
@@ -581,10 +581,14 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Demand for the cycle is derived from confirmed orders and distributors' Best Estimate, family by family</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr"/>
+          <t>Requirement collected plant-wise; demand derived from confirmed orders and distributors' Best Estimate, family by family</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Siddharth - Planning (dedicated resource needed)</t>
+        </is>
+      </c>
       <c r="D4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
@@ -628,204 +632,228 @@
       <c r="D8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="n"/>
+      <c r="A9" s="7" t="n"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Published as a rolling size-by-week program with per-family open/closed status and order cut-offs</t>
+          <t>Schedule planned and material ageing tracked against the plan</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr"/>
       <c r="D9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>2. RM Opportunity</t>
-        </is>
-      </c>
+      <c r="A10" s="8" t="n"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>RM opportunity created in SFDC</t>
+          <t>Published as a rolling size-by-week program with per-family open/closed status and order cut-offs</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr"/>
       <c r="D10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="n"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>2. Quality &amp; Source Approval</t>
+        </is>
+      </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>SLO created</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr"/>
+          <t>Incoming quality process set up</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Arijit - Quality (associate role needed)</t>
+        </is>
+      </c>
       <c r="D11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>3. Order Creation</t>
-        </is>
-      </c>
+      <c r="A12" s="8" t="n"/>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Supply chain reviews the SLO and identifies the plant that will fulfil it</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr"/>
+          <t>New TDC (technical delivery condition) and source approval for material sources</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Arijit - Quality</t>
+        </is>
+      </c>
       <c r="D12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n"/>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>3. RM Opportunity</t>
+        </is>
+      </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Order is created against that plant</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr"/>
+          <t>RM opportunity created in SFDC</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Atul - Sales</t>
+        </is>
+      </c>
       <c r="D13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n"/>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>SO generated in SFDC, linked back to the SLO and the RM opportunity</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr"/>
+          <t>SLO created</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Atul - Sales</t>
+        </is>
+      </c>
       <c r="D14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>4. Material Readiness &amp; Invoice Amount Check</t>
+          <t>4. Order Creation</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Category team checks whether the ordered material is ready/available against the SO</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr"/>
+          <t>Supply chain reviews the SLO and identifies the plant that will fulfil it</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Sanjay Jha - Operations</t>
+        </is>
+      </c>
       <c r="D15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
       <c r="B16" s="5" t="inlineStr">
         <is>
+          <t>Order is created against that plant</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Sanjay Jha - Operations</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>SO generated in SFDC, linked back to the SLO and the RM opportunity</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Sanjay Jha - Operations</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>5. CM Plant Contracting &amp; Payment</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Contracting and payment terms agreed with CM (contract manufacturing) plants</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Vinay (interview done, confirmation pending)</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>6. Material Readiness &amp; Invoice Amount Check</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Category team checks whether the ordered material is ready/available against the SO</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Debdeep - Planning &amp; Sanjay Jha (CM side) (dedicated resource needed)</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="n"/>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
           <t>Supply team works out the amount to be collected for the invoice, based on the SO and material readiness</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr"/>
-      <c r="D16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="n"/>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Category and Supply teams coordinate manually (call/email) — no dedicated system today; this is the main gap in the process</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="inlineStr"/>
-      <c r="D17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="n"/>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Debdeep - Planning &amp; Sanjay Jha (CM side) (dedicated resource needed)</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Category and Supply teams coordinate manually (call/email) — no dedicated tracker or system today; this is the main gap in the process</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Debdeep - Planning &amp; Sanjay Jha (CM side) (dedicated resource needed)</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Order becomes eligible for invoicing once both readiness and invoice amount are confirmed</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr"/>
-      <c r="D18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>5. Invoicing</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Invoice raised; invoice visibility available</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr"/>
-      <c r="D19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>6. Coil Inward</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Coil inwarded once invoiced — pipeline process begins</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>Zoho Creator (future)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Mother HR coil registered: date, plant, coil ID, grade, thickness, width, weight, cost price, PO number</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr"/>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Zoho Creator (future)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>7. Slitting</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Mother coil picked; baby-coil widths entered</t>
-        </is>
-      </c>
       <c r="C22" s="6" t="inlineStr"/>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>Zoho Creator (future)</t>
-        </is>
-      </c>
+      <c r="D22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="n"/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>7. Invoicing → Production</t>
+        </is>
+      </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Weight &amp; cost split proportionally across baby coils</t>
+          <t>Invoicing — invoice raised; invoice visibility available</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr"/>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>Zoho Creator (future)</t>
-        </is>
-      </c>
+      <c r="D23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>8. Production</t>
-        </is>
-      </c>
+      <c r="A24" s="7" t="n"/>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Date, SKU and pieces recorded</t>
+          <t>Coil Inward — coil inwarded once invoiced; pipeline process begins</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr"/>
@@ -836,10 +864,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="n"/>
+      <c r="A25" s="7" t="n"/>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>FIFO suggestion reviewed; actual coil allocation confirmed/edited manually</t>
+          <t>Coil Inward — mother HR coil registered: date, plant, coil ID, grade, thickness, width, weight, cost price, PO number</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr"/>
@@ -850,14 +878,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>9. Dispatch</t>
-        </is>
-      </c>
+      <c r="A26" s="7" t="n"/>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Daily Sales Excel uploaded</t>
+          <t>Slitting — mother coil picked; baby-coil widths entered</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr"/>
@@ -868,10 +892,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="n"/>
+      <c r="A27" s="7" t="n"/>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Rows grouped into one dispatch per date × vehicle; coil trace inherited from Production</t>
+          <t>Slitting — weight &amp; cost split proportionally across baby coils</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr"/>
@@ -882,14 +906,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>10. Sales / Reporting</t>
-        </is>
-      </c>
+      <c r="A28" s="7" t="n"/>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Confirmed / Non-confirmed / Pending to Dispatch / Invoiced tracked per distributor</t>
+          <t>Production — date, SKU and pieces recorded</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr"/>
@@ -903,7 +923,7 @@
       <c r="A29" s="8" t="n"/>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Best Estimate maintained; MTD &amp; daily reports generated</t>
+          <t>Production — FIFO suggestion reviewed; actual coil allocation confirmed/edited manually</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr"/>
@@ -916,98 +936,226 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>11. Campaign Monitoring</t>
+          <t>8. Dispatch</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
+          <t>Daily Sales Excel uploaded</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr"/>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Creator (future)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Rows grouped into one dispatch per date × vehicle; coil trace inherited from Production</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr"/>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Creator (future)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>9. Sales / Reporting</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed / Non-confirmed / Pending to Dispatch / Invoiced tracked per distributor</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr"/>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Creator (future)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Best Estimate maintained; MTD &amp; daily reports generated</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Creator (future)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>10. Campaign Monitoring</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
           <t>Campaign progress tracked weekly — planned vs produced, by SKU</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr"/>
-      <c r="D30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="n"/>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr"/>
+      <c r="D34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="n"/>
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>Deferred families and idle mill-days flagged</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr"/>
-      <c r="D31" s="6" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="n"/>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr"/>
+      <c r="D35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Distributors to chase decided — confirmed orders where payment hasn't come in</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr"/>
-      <c r="D32" s="6" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="C36" s="6" t="inlineStr"/>
+      <c r="D36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>11. Month-End Reconciliation &amp; Settlement</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Reconcile the month — pull One Helix exports, run FIFO/Thickness close, commit to masters</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Siddharth</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n"/>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Book the settlement — record Net CN/DN</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Siddharth</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Books</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>• Step 4 is the main gap: no system exists today for the Category/Supply team's material-readiness and invoice-amount check — it is coordinated manually.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="11" t="inlineStr">
-        <is>
-          <t>• Steps 6–10 run in this app (the JSW Pipes &amp; Tubes Inventory system) today; System/Software shows the planned future system, Zoho Creator.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>• Step 6 is the main gap: no system exists today for the Category/Supply team's material-readiness and invoice-amount check — it is coordinated manually and needs "a proper tracker and mechanism." It requires coordination with plants, category team and supply team; the role also needs an understanding of credit and finance, and depends on fund availability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>• Step 1's "material ageing" sub-step has no owner named — a second, smaller gap alongside step 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>• Steps 2, 3, 4, 5, 6 and 11 carry named owners, taken as given from the team's responsibility sheet — including two pending items: the Quality associate role in step 2 is not yet filled, and Vinay's role in step 5 is pending confirmation (interview done, status to be checked).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>• Steps 2 (Quality &amp; Source Approval) and 5 (CM Plant Contracting &amp; Payment) are new steps inferred from that responsibility sheet — positioned here as the most logical fit. Reposition if they sit elsewhere in the actual flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>• Step 7's Coil Inward / Slitting / Production sub-steps, plus steps 8 (Dispatch) and 9 (Sales/Reporting), run in this app (the JSW Pipes &amp; Tubes Inventory system) today; System/Software shows the planned future system, Zoho Creator. The Invoicing sub-step itself is SFDC-side, not this app, so it is left blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="11" t="inlineStr">
         <is>
           <t>• Campaign Planning and Campaign Monitoring reflect the P&amp;T Command Centre design research (.scratch/pt-os-research/) — a screen-level design/prototype, not yet built as live software.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>• SLO and SO are used as given; not expanded here since their exact meaning wasn't specified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="11" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>• SLO, SO and TDC are used as given; not expanded beyond "technical delivery condition" for TDC, since exact meanings weren't specified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t>• Person and System / Software are blank except where noted — for process owners to complete. Yellow cells mark where entry is expected.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="20">
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A4:A10"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A23:A29"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A37:A38"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="A37:D37"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="A4:A9"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A38:D38"/>
-    <mergeCell ref="A39:D39"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A15:A18"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A46:D46"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A47:D47"/>
+    <mergeCell ref="A42:D42"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A30:A31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix Vinay's step: restore dropped dedicated-resource tag, split into 2 sub-steps
Book_82's row 7 (Vinay, CM plant contracting) has the same "Dedicated
resource" Support Required value as Siddharth's and Debdeep's rows,
but it was dropped when step 5 was first written. Restored it, and
split the single "Contracting and payment" line into its two
component sub-steps to match the granularity given to every other
person's row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J9TXredfbUcJ8vSi96NRVo
</commit_message>
<xml_diff>
--- a/docs/PROCESS-MAP.xlsx
+++ b/docs/PROCESS-MAP.xlsx
@@ -134,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -156,9 +156,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -528,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -762,46 +759,46 @@
       <c r="D17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>5. CM Plant Contracting &amp; Payment</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Contracting and payment terms agreed with CM (contract manufacturing) plants</t>
+          <t>Contract terms negotiated with CM (contract manufacturing) plants</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Vinay (interview done, confirmation pending)</t>
+          <t>Vinay (dedicated resource; interview done, confirmation pending)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Payment terms agreed with CM plants</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Vinay (dedicated resource; interview done, confirmation pending)</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>6. Material Readiness &amp; Invoice Amount Check</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Category team checks whether the ordered material is ready/available against the SO</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Debdeep - Planning &amp; Sanjay Jha (CM side) (dedicated resource needed)</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="n"/>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Supply team works out the amount to be collected for the invoice, based on the SO and material readiness</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -815,59 +812,59 @@
       <c r="A21" s="7" t="n"/>
       <c r="B21" s="5" t="inlineStr">
         <is>
+          <t>Supply team works out the amount to be collected for the invoice, based on the SO and material readiness</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Debdeep - Planning &amp; Sanjay Jha (CM side) (dedicated resource needed)</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n"/>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
           <t>Category and Supply teams coordinate manually (call/email) — no dedicated tracker or system today; this is the main gap in the process</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Debdeep - Planning &amp; Sanjay Jha (CM side) (dedicated resource needed)</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="n"/>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Order becomes eligible for invoicing once both readiness and invoice amount are confirmed</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr"/>
-      <c r="D22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>7. Invoicing → Production</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Invoicing — invoice raised; invoice visibility available</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr"/>
       <c r="D23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="n"/>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>7. Invoicing → Production</t>
+        </is>
+      </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Coil Inward — coil inwarded once invoiced; pipeline process begins</t>
+          <t>Invoicing — invoice raised; invoice visibility available</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr"/>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>Zoho Creator (future)</t>
-        </is>
-      </c>
+      <c r="D24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Coil Inward — mother HR coil registered: date, plant, coil ID, grade, thickness, width, weight, cost price, PO number</t>
+          <t>Coil Inward — coil inwarded once invoiced; pipeline process begins</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr"/>
@@ -881,7 +878,7 @@
       <c r="A26" s="7" t="n"/>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Slitting — mother coil picked; baby-coil widths entered</t>
+          <t>Coil Inward — mother HR coil registered: date, plant, coil ID, grade, thickness, width, weight, cost price, PO number</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr"/>
@@ -895,7 +892,7 @@
       <c r="A27" s="7" t="n"/>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Slitting — weight &amp; cost split proportionally across baby coils</t>
+          <t>Slitting — mother coil picked; baby-coil widths entered</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr"/>
@@ -909,7 +906,7 @@
       <c r="A28" s="7" t="n"/>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Production — date, SKU and pieces recorded</t>
+          <t>Slitting — weight &amp; cost split proportionally across baby coils</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr"/>
@@ -920,10 +917,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="n"/>
+      <c r="A29" s="7" t="n"/>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Production — FIFO suggestion reviewed; actual coil allocation confirmed/edited manually</t>
+          <t>Production — date, SKU and pieces recorded</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr"/>
@@ -934,14 +931,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>8. Dispatch</t>
-        </is>
-      </c>
+      <c r="A30" s="8" t="n"/>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Daily Sales Excel uploaded</t>
+          <t>Production — FIFO suggestion reviewed; actual coil allocation confirmed/edited manually</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr"/>
@@ -952,10 +945,14 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="n"/>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>8. Dispatch</t>
+        </is>
+      </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Rows grouped into one dispatch per date × vehicle; coil trace inherited from Production</t>
+          <t>Daily Sales Excel uploaded</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr"/>
@@ -966,14 +963,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>9. Sales / Reporting</t>
-        </is>
-      </c>
+      <c r="A32" s="8" t="n"/>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Confirmed / Non-confirmed / Pending to Dispatch / Invoiced tracked per distributor</t>
+          <t>Rows grouped into one dispatch per date × vehicle; coil trace inherited from Production</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr"/>
@@ -984,10 +977,14 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="n"/>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>9. Sales / Reporting</t>
+        </is>
+      </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Best Estimate maintained; MTD &amp; daily reports generated</t>
+          <t>Confirmed / Non-confirmed / Pending to Dispatch / Invoiced tracked per distributor</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr"/>
@@ -998,164 +995,179 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Best Estimate maintained; MTD &amp; daily reports generated</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr"/>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Zoho Creator (future)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>10. Campaign Monitoring</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>Campaign progress tracked weekly — planned vs produced, by SKU</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr"/>
-      <c r="D34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="n"/>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>Deferred families and idle mill-days flagged</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr"/>
       <c r="D35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="n"/>
+      <c r="A36" s="7" t="n"/>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Distributors to chase decided — confirmed orders where payment hasn't come in</t>
+          <t>Deferred families and idle mill-days flagged</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr"/>
       <c r="D36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Distributors to chase decided — confirmed orders where payment hasn't come in</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr"/>
+      <c r="D37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>11. Month-End Reconciliation &amp; Settlement</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>Reconcile the month — pull One Helix exports, run FIFO/Thickness close, commit to masters</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>Siddharth</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>Excel</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="8" t="n"/>
-      <c r="B38" s="5" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="8" t="n"/>
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Book the settlement — record Net CN/DN</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>Siddharth</t>
         </is>
       </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>Zoho Books</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="11" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>• Step 6 is the main gap: no system exists today for the Category/Supply team's material-readiness and invoice-amount check — it is coordinated manually and needs "a proper tracker and mechanism." It requires coordination with plants, category team and supply team; the role also needs an understanding of credit and finance, and depends on fund availability.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>• Step 1's "material ageing" sub-step has no owner named — a second, smaller gap alongside step 6.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>• Steps 2, 3, 4, 5, 6 and 11 carry named owners, taken as given from the team's responsibility sheet — including two pending items: the Quality associate role in step 2 is not yet filled, and Vinay's role in step 5 is pending confirmation (interview done, status to be checked).</t>
-        </is>
-      </c>
-    </row>
     <row r="44">
-      <c r="A44" s="11" t="inlineStr">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>• Steps 2, 3, 4, 5, 6 and 11 carry named owners, taken as given from the team's responsibility sheet — including three pending items: the Quality associate role in step 2 is not yet filled, step 5 (Vinay) is flagged as a dedicated resource with confirmation still pending (interview done, status to be checked), and step 6 also needs a dedicated resource.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
         <is>
           <t>• Steps 2 (Quality &amp; Source Approval) and 5 (CM Plant Contracting &amp; Payment) are new steps inferred from that responsibility sheet — positioned here as the most logical fit. Reposition if they sit elsewhere in the actual flow.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="11" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
         <is>
           <t>• Step 7's Coil Inward / Slitting / Production sub-steps, plus steps 8 (Dispatch) and 9 (Sales/Reporting), run in this app (the JSW Pipes &amp; Tubes Inventory system) today; System/Software shows the planned future system, Zoho Creator. The Invoicing sub-step itself is SFDC-side, not this app, so it is left blank.</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="11" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>• Campaign Planning and Campaign Monitoring reflect the P&amp;T Command Centre design research (.scratch/pt-os-research/) — a screen-level design/prototype, not yet built as live software.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="11" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>• SLO, SO and TDC are used as given; not expanded beyond "technical delivery condition" for TDC, since exact meanings weren't specified.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="11" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
         <is>
           <t>• Person and System / Software are blank except where noted — for process owners to complete. Yellow cells mark where entry is expected.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A35:A37"/>
     <mergeCell ref="A4:A10"/>
-    <mergeCell ref="A34:A36"/>
     <mergeCell ref="A48:D48"/>
-    <mergeCell ref="A23:A29"/>
     <mergeCell ref="A15:A17"/>
-    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A18:A19"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A32:A33"/>
     <mergeCell ref="A45:D45"/>
     <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="A24:A30"/>
     <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="A31:A32"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A47:D47"/>
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A30:A31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>